<commit_message>
Update sources section with full reference list from kaynaklar.xlsx
</commit_message>
<xml_diff>
--- a/kaynaklar.xlsx
+++ b/kaynaklar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NusretAgayani\Desktop\grafikler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B4F6A3-950E-4749-851D-FCE5589A4C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C8F1CA-AA40-43F4-A6CA-447232E75935}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="111">
   <si>
     <t>https://arabcenterdc.org/resource/the-estimated-cost-of-the-gaza-war-on-the-israeli-economy/</t>
   </si>
@@ -78,12 +78,6 @@
     <t>https://www.reuters.com/world/middle-east/damage-israeli-economy-iran-war-could-top-29-billion-week-ministry-says-2026-03-04/</t>
   </si>
   <si>
-    <t>Reuters – Yeni kaynak</t>
-  </si>
-  <si>
-    <t>Daily Sabah – Mevcut kaynak (aynı veriyi doğruluyor)</t>
-  </si>
-  <si>
     <t>500+ balistik &amp; seyir füzesi atılması</t>
   </si>
   <si>
@@ -114,39 +108,18 @@
     <t>100.000 yedek askerin tahmini maliyeti</t>
   </si>
   <si>
-    <t>Arab Center DC – Mevcut + Yeni kaynak (maliyet hesabı)</t>
-  </si>
-  <si>
     <t>Gaz sahaları ve rafineri kapatılması (saldırı sonrası)</t>
   </si>
   <si>
-    <t>Argus Media – Mevcut + Yeni kaynak</t>
-  </si>
-  <si>
-    <t>İran füzesinin rafineriye isabeti ve hasar detayı</t>
-  </si>
-  <si>
-    <t>https://www.calcalistech.com/ctechnews/article/le511t25l</t>
-  </si>
-  <si>
-    <t>Calcalist – Mevcut + Yeni kaynak</t>
-  </si>
-  <si>
     <t>12 günlük savaşta askeri maliyet (stok yenileme, mühimmat, rezervist maaşları, savunma sistemi bakımı)</t>
   </si>
   <si>
     <t>Kapanmadan dolayı oluşan maliyet: 3 milyar $/hafta</t>
   </si>
   <si>
-    <t>Reuters – Toplam maliyetin bir parçası olarak kapanma</t>
-  </si>
-  <si>
     <t>Günlük yüzlerce milyon dolarlık savaş maliyeti</t>
   </si>
   <si>
-    <t>WSJ – Mevcut kaynak</t>
-  </si>
-  <si>
     <t>Turizm rakamları, savaş sonrası turizm canlandırma çalışmaları</t>
   </si>
   <si>
@@ -355,13 +328,46 @@
   </si>
   <si>
     <t>https://tr.investing.com/</t>
+  </si>
+  <si>
+    <t>TOPLAM SAVAŞ MALİYETİ</t>
+  </si>
+  <si>
+    <t>Savaşın toplam maliyeti: ~95 milyar $ (İsrail GSYH'sinin %18'i). Savunma harcamaları (~45 milyar $), altyapı onarımı (~20 milyar $), askeri teçhizat yenileme (~15 milyar $), yaralı rehabilitasyonu ve tazminatlar (~15 milyar $) dahil.</t>
+  </si>
+  <si>
+    <t>https://jcfa.org/article/the-israeli-economy-during-the-october-7-2023-war-and-its-aftermath/</t>
+  </si>
+  <si>
+    <t>Reuters – Haftalık ekonomik kapanma maliyeti</t>
+  </si>
+  <si>
+    <t>Daily Sabah – Haftalık ekonomik kapanma maliyeti</t>
+  </si>
+  <si>
+    <t>Arab Center DC – Yedek asker maliyet hesabı</t>
+  </si>
+  <si>
+    <t>Argus Media – Gaz sahaları ve rafineri kapatılması</t>
+  </si>
+  <si>
+    <t>Calcalist – 12 günlük savaş askeri maliyet analizi</t>
+  </si>
+  <si>
+    <t>WSJ – Günlük yüzlerce milyon dolarlık savaş maliyeti</t>
+  </si>
+  <si>
+    <t>Reuters – Kapanma kaynaklı haftalık maliyet</t>
+  </si>
+  <si>
+    <t>JCFA – Toplam savaş maliyeti ~95 milyar $</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -414,6 +420,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF2E75B6"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -505,7 +517,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -525,6 +537,12 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Köprü" xfId="1" builtinId="8"/>
@@ -828,7 +846,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.5703125" customWidth="1"/>
@@ -853,7 +871,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -868,7 +886,7 @@
         <v>15</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>16</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -880,12 +898,12 @@
         <v>1</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>17</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -894,30 +912,30 @@
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>18</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -926,40 +944,40 @@
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
       <c r="B9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>0</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="4" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="D11" s="6"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -968,423 +986,434 @@
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="11" t="s">
         <v>9</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>30</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>33</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="D14" s="6"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="4" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="D15" s="6"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
-      <c r="B16" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D16" s="6"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
+        <v>81</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>7</v>
+        <v>28</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>33</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="4" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>36</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
-      <c r="B20" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>38</v>
-      </c>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
+        <v>82</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
       <c r="B22" s="4" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
       <c r="B23" s="4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
-      <c r="B24" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>47</v>
-      </c>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
+        <v>83</v>
+      </c>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="10"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="9">
         <v>2024</v>
       </c>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
+      <c r="B26" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="4" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
-      <c r="B28" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="10"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>2025</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
+      <c r="B29" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
       <c r="B30" s="4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
-      <c r="B31" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>59</v>
-      </c>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="9">
         <v>2026</v>
       </c>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
+      <c r="B32" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>61</v>
+        <v>54</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>55</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
-      <c r="B34" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>65</v>
-      </c>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
+        <v>84</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
       <c r="B36" s="4" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="4" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
       <c r="B38" s="4" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="4" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
-      <c r="B40" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>74</v>
-      </c>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
+        <v>85</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C41" s="11" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B42" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C42" s="11" t="s">
-        <v>81</v>
+        <v>73</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B43" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C43" s="12" t="s">
-        <v>83</v>
+        <v>75</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B44" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C44" s="13" t="s">
-        <v>85</v>
-      </c>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
+        <v>86</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D45" s="15"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
-      <c r="B46" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C46" s="16" t="s">
-        <v>97</v>
-      </c>
-      <c r="D46" s="15"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B47" t="s">
+        <v>90</v>
+      </c>
+      <c r="C47" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B49" t="s">
+        <v>93</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>95</v>
+      </c>
+      <c r="C50" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B52" t="s">
         <v>98</v>
       </c>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
+      <c r="C52" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="C48" s="13" t="s">
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54" s="17" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="7" t="s">
+      <c r="B54" s="18"/>
+      <c r="C54" s="18"/>
+      <c r="D54" s="18"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55" s="19"/>
+      <c r="B55" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B50" t="s">
+      <c r="C55" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="C50" s="13" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B51" t="s">
-        <v>104</v>
-      </c>
-      <c r="C51" s="13" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="B52" s="8"/>
-      <c r="C52" s="8"/>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B53" t="s">
-        <v>107</v>
-      </c>
-      <c r="C53" s="13" t="s">
-        <v>108</v>
+      <c r="D55" s="21" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C11" r:id="rId1" xr:uid="{FC0D0975-495B-4EAB-8617-AA5FD16029C3}"/>
-    <hyperlink ref="C15" r:id="rId2" xr:uid="{1E5CF3F5-7279-49B9-8DF9-E1D8DB865C05}"/>
-    <hyperlink ref="C16" r:id="rId3" xr:uid="{00B7A003-227A-4A7B-8C35-14B61ECF965F}"/>
-    <hyperlink ref="C42" r:id="rId4" xr:uid="{01BAF331-3686-46EB-9B68-5F9C5B22E9B7}"/>
-    <hyperlink ref="C43" r:id="rId5" xr:uid="{F7CEB547-8FCD-491A-9E4B-F3B4F1E119C9}"/>
-    <hyperlink ref="C44" r:id="rId6" xr:uid="{97009C7C-897F-4B28-A19D-2D4199CD7CE6}"/>
-    <hyperlink ref="C18" r:id="rId7" xr:uid="{6B00FE96-9593-4BC8-8AB0-9EE27DC04AE3}"/>
-    <hyperlink ref="C34" r:id="rId8" xr:uid="{375604BA-6F58-4406-A957-F12EEF425F46}"/>
-    <hyperlink ref="C46" r:id="rId9" xr:uid="{97B7EF4E-86D4-464C-91F8-3488B247730D}"/>
-    <hyperlink ref="C48" r:id="rId10" xr:uid="{77633BB4-648C-4223-94AF-BD70D31C5DCB}"/>
-    <hyperlink ref="C50" r:id="rId11" xr:uid="{43FE0547-8B69-4A18-9E37-08DD4659F5EE}"/>
-    <hyperlink ref="C51" r:id="rId12" xr:uid="{630FF9C7-07C0-43AA-84D7-2E6B7E3F5C0F}"/>
-    <hyperlink ref="C53" r:id="rId13" xr:uid="{7AE4EDE5-F892-4E26-A0EA-1C04C049D876}"/>
+    <hyperlink ref="C14" r:id="rId2" xr:uid="{1E5CF3F5-7279-49B9-8DF9-E1D8DB865C05}"/>
+    <hyperlink ref="C15" r:id="rId3" xr:uid="{00B7A003-227A-4A7B-8C35-14B61ECF965F}"/>
+    <hyperlink ref="C41" r:id="rId4" xr:uid="{01BAF331-3686-46EB-9B68-5F9C5B22E9B7}"/>
+    <hyperlink ref="C42" r:id="rId5" xr:uid="{F7CEB547-8FCD-491A-9E4B-F3B4F1E119C9}"/>
+    <hyperlink ref="C43" r:id="rId6" xr:uid="{97009C7C-897F-4B28-A19D-2D4199CD7CE6}"/>
+    <hyperlink ref="C17" r:id="rId7" xr:uid="{6B00FE96-9593-4BC8-8AB0-9EE27DC04AE3}"/>
+    <hyperlink ref="C33" r:id="rId8" xr:uid="{375604BA-6F58-4406-A957-F12EEF425F46}"/>
+    <hyperlink ref="C45" r:id="rId9" xr:uid="{97B7EF4E-86D4-464C-91F8-3488B247730D}"/>
+    <hyperlink ref="C47" r:id="rId10" xr:uid="{77633BB4-648C-4223-94AF-BD70D31C5DCB}"/>
+    <hyperlink ref="C49" r:id="rId11" xr:uid="{43FE0547-8B69-4A18-9E37-08DD4659F5EE}"/>
+    <hyperlink ref="C50" r:id="rId12" xr:uid="{630FF9C7-07C0-43AA-84D7-2E6B7E3F5C0F}"/>
+    <hyperlink ref="C52" r:id="rId13" xr:uid="{7AE4EDE5-F892-4E26-A0EA-1C04C049D876}"/>
+    <hyperlink ref="C13" r:id="rId14" xr:uid="{DDD4EDDC-5D9B-4E85-B37C-7AE7005525FD}"/>
+    <hyperlink ref="C55" r:id="rId15" xr:uid="{30DA78A7-EC78-4033-BD40-2DD90975FE18}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>